<commit_message>
Docs: guia informa que produtos com mais de um endereço são importados e exibidos por inteiro
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmX7GPsvZca49dKD49DNem
</commit_message>
<xml_diff>
--- a/docs/modelo-entrada-manual.xlsx
+++ b/docs/modelo-entrada-manual.xlsx
@@ -397,12 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="70.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,9 +531,23 @@
         <v>C039</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PB310</v>
+      </c>
+      <c r="B10">
+        <v>24</v>
+      </c>
+      <c r="C10" t="str">
+        <v>K Blend Gel Deslizante Neutro 50g Pepper Blend</v>
+      </c>
+      <c r="D10" t="str">
+        <v>U331, VERT-U10-CX16</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>